<commit_message>
Refined figures for rev1
</commit_message>
<xml_diff>
--- a/auxiliary_data/Citable_documents_per_country.xlsx
+++ b/auxiliary_data/Citable_documents_per_country.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20411"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meurerst\git\anonymization-review\auxiliary_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28928F3-797D-46C4-B2C5-83AE5D3C343B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D2F521-46B7-4C00-BDBD-E668D38EBDAB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="14724" windowHeight="4428" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Citable_documents_per_country" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="245">
   <si>
     <t>Name (Country)</t>
   </si>
@@ -752,6 +752,9 @@
   </si>
   <si>
     <t>Russia</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -770,6 +773,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1114,7 +1118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G238"/>
+  <dimension ref="A1:G240"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -6423,6 +6427,35 @@
         <v>2133</v>
       </c>
     </row>
+    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>244</v>
+      </c>
+      <c r="B240">
+        <f t="shared" ref="B240:F240" si="0">SUM(B2:B238)</f>
+        <v>1024350</v>
+      </c>
+      <c r="C240">
+        <f t="shared" si="0"/>
+        <v>1084371</v>
+      </c>
+      <c r="D240">
+        <f t="shared" si="0"/>
+        <v>1220919</v>
+      </c>
+      <c r="E240">
+        <f t="shared" si="0"/>
+        <v>1390423</v>
+      </c>
+      <c r="F240">
+        <f t="shared" si="0"/>
+        <v>1433601</v>
+      </c>
+      <c r="G240">
+        <f>SUM(G2:G238)</f>
+        <v>6153664</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed unknown origin records, removed gini, added datatype evaluation
</commit_message>
<xml_diff>
--- a/auxiliary_data/Citable_documents_per_country.xlsx
+++ b/auxiliary_data/Citable_documents_per_country.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meurerst\git\anonymization-review\auxiliary_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D2F521-46B7-4C00-BDBD-E668D38EBDAB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5161E436-B495-417A-88E7-5B450C402976}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="14724" windowHeight="4428" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="244">
   <si>
     <t>Name (Country)</t>
   </si>
@@ -752,9 +752,6 @@
   </si>
   <si>
     <t>Russia</t>
-  </si>
-  <si>
-    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -1118,7 +1115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G240"/>
+  <dimension ref="A1:G238"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -6427,35 +6424,6 @@
         <v>2133</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A240" t="s">
-        <v>244</v>
-      </c>
-      <c r="B240">
-        <f t="shared" ref="B240:F240" si="0">SUM(B2:B238)</f>
-        <v>1024350</v>
-      </c>
-      <c r="C240">
-        <f t="shared" si="0"/>
-        <v>1084371</v>
-      </c>
-      <c r="D240">
-        <f t="shared" si="0"/>
-        <v>1220919</v>
-      </c>
-      <c r="E240">
-        <f t="shared" si="0"/>
-        <v>1390423</v>
-      </c>
-      <c r="F240">
-        <f t="shared" si="0"/>
-        <v>1433601</v>
-      </c>
-      <c r="G240">
-        <f>SUM(G2:G238)</f>
-        <v>6153664</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>